<commit_message>
VE: corregir comparativa vs Aura (total Aura calculado del Excel real)
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01PL4fade9uMUQLM1tmUvUUs
</commit_message>
<xml_diff>
--- a/URBANSIP/catalogo/VIVIENDAS_ECONOMICAS/presupuesto/VE_vs_Aura_Comparativa.xlsx
+++ b/URBANSIP/catalogo/VIVIENDAS_ECONOMICAS/presupuesto/VE_vs_Aura_Comparativa.xlsx
@@ -17,7 +17,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="8">
+  <fonts count="2">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -27,43 +27,14 @@
     </font>
     <font>
       <b val="1"/>
-      <sz val="12"/>
-    </font>
-    <font>
-      <b val="1"/>
-      <color rgb="00FFFFFF"/>
-    </font>
-    <font>
-      <color rgb="00FF0000"/>
-    </font>
-    <font>
-      <color rgb="0000B050"/>
-    </font>
-    <font>
-      <b val="1"/>
-      <color rgb="000066CC"/>
-      <sz val="11"/>
-    </font>
-    <font>
-      <b val="1"/>
-    </font>
-    <font>
-      <i val="1"/>
-      <sz val="9"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="2">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00366092"/>
-        <bgColor rgb="00366092"/>
-      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -78,15 +49,9 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -452,299 +417,475 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E27"/>
+  <dimension ref="A1:E25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="50" customWidth="1" min="1" max="1"/>
-    <col width="16" customWidth="1" min="2" max="2"/>
-    <col width="16" customWidth="1" min="3" max="3"/>
-    <col width="16" customWidth="1" min="4" max="4"/>
-    <col width="16" customWidth="1" min="5" max="5"/>
+    <col width="52" customWidth="1" min="1" max="1"/>
+    <col width="20" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="18" customWidth="1" min="4" max="4"/>
+    <col width="8" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>COMPARATIVA: VIVIENDAS ECONÓMICAS vs AURA ESENCIAL</t>
+          <t>Rubro</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Aura Esencial (USD)</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>VE (USD)</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Diferencia (USD)</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Dif. %</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Fundación (vigas, contrapisos, carpeta)</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>1888</v>
+      </c>
+      <c r="C2" t="n">
+        <v>1888</v>
+      </c>
+      <c r="D2" t="n">
+        <v>0</v>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>0%</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="2" t="inlineStr">
-        <is>
-          <t>Concepto</t>
-        </is>
-      </c>
-      <c r="B3" s="2" t="inlineStr">
-        <is>
-          <t>Aura Esencial</t>
-        </is>
-      </c>
-      <c r="C3" s="2" t="inlineStr">
-        <is>
-          <t>VE Económica</t>
-        </is>
-      </c>
-      <c r="D3" s="2" t="inlineStr">
-        <is>
-          <t>Diferencia (USD)</t>
-        </is>
-      </c>
-      <c r="E3" s="2" t="inlineStr">
-        <is>
-          <t>Diferencia (%)</t>
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Mantenimiento de obra</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>426</v>
+      </c>
+      <c r="C3" t="n">
+        <v>426</v>
+      </c>
+      <c r="D3" t="n">
+        <v>0</v>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>0%</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Costo Materiales (USD)</t>
+          <t>Kit SIP + flete + sellado + dinteles</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>-22705</v>
+        <v>18830</v>
       </c>
       <c r="C4" t="n">
-        <v>33747</v>
-      </c>
-      <c r="D4" s="3" t="n">
-        <v>56452</v>
-      </c>
-      <c r="E4" s="4" t="inlineStr">
-        <is>
-          <t>-248.6%</t>
+        <v>18830</v>
+      </c>
+      <c r="D4" t="n">
+        <v>0</v>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>-0%</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Mano de Obra (USD)</t>
+          <t>Durlock</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>24820</v>
+        <v>892</v>
       </c>
       <c r="C5" t="n">
-        <v>24820</v>
-      </c>
-      <c r="D5" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="E5" s="4" t="inlineStr">
-        <is>
-          <t>0.0%</t>
+        <v>892</v>
+      </c>
+      <c r="D5" t="n">
+        <v>0</v>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>-0%</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>COSTO TOTAL (USD)</t>
+          <t>Revestimiento exterior (siding LP / placa cementicia)</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>2114</v>
+        <v>1595</v>
       </c>
       <c r="C6" t="n">
-        <v>58567</v>
-      </c>
-      <c r="D6" s="3" t="n">
-        <v>56453</v>
-      </c>
-      <c r="E6" s="3" t="inlineStr">
-        <is>
-          <t>2670.4%</t>
+        <v>839</v>
+      </c>
+      <c r="D6" t="n">
+        <v>-756</v>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>-47%</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Costo por m² (USD)</t>
+          <t>Techo (chapa C25 / galvanizada)</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>612</v>
+        <v>2280</v>
       </c>
       <c r="C7" t="n">
-        <v>802</v>
-      </c>
-      <c r="D7" s="3" t="n">
-        <v>190</v>
-      </c>
-      <c r="E7" s="3" t="inlineStr">
-        <is>
-          <t>31.0%</t>
+        <v>906</v>
+      </c>
+      <c r="D7" t="n">
+        <v>-1374</v>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>-60%</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Canaletas y zinguería</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>1319</v>
+      </c>
+      <c r="C8" t="n">
+        <v>1319</v>
+      </c>
+      <c r="D8" t="n">
+        <v>0</v>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>0%</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Sanitaria (materiales + artefactos + extractor)</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
+        <v>1325</v>
+      </c>
+      <c r="C9" t="n">
+        <v>677</v>
+      </c>
+      <c r="D9" t="n">
+        <v>-648</v>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>-49%</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Eléctrica (materiales)</t>
+        </is>
+      </c>
+      <c r="B10" t="n">
+        <v>2090</v>
+      </c>
+      <c r="C10" t="n">
+        <v>2090</v>
+      </c>
+      <c r="D10" t="n">
+        <v>0</v>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>0%</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="5" t="inlineStr">
-        <is>
-          <t>CAMBIOS REALIZADOS EN VE:</t>
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Puertas y herrajes</t>
+        </is>
+      </c>
+      <c r="B11" t="n">
+        <v>1750</v>
+      </c>
+      <c r="C11" t="n">
+        <v>818</v>
+      </c>
+      <c r="D11" t="n">
+        <v>-932</v>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>-53%</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Aberturas aluminio</t>
+        </is>
+      </c>
+      <c r="B12" t="n">
+        <v>3226</v>
+      </c>
+      <c r="C12" t="n">
+        <v>1613</v>
+      </c>
+      <c r="D12" t="n">
+        <v>-1613</v>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>-50%</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Siding LP $18.055/m² → Placa cementicia $9.500/m²</t>
-        </is>
-      </c>
-      <c r="B13" t="inlineStr">
-        <is>
-          <t>−47%</t>
-        </is>
-      </c>
-      <c r="C13" t="inlineStr">
-        <is>
-          <t>-1.172 USD</t>
+          <t>Pisos y zócalos</t>
+        </is>
+      </c>
+      <c r="B13" t="n">
+        <v>2962</v>
+      </c>
+      <c r="C13" t="n">
+        <v>1803</v>
+      </c>
+      <c r="D13" t="n">
+        <v>-1159</v>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>-39%</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Chapa C25 zinc $45.303/m² → Galvanizado $18.000/m²</t>
-        </is>
-      </c>
-      <c r="B14" t="inlineStr">
-        <is>
-          <t>−60%</t>
-        </is>
-      </c>
-      <c r="C14" t="inlineStr">
-        <is>
-          <t>-2.124 USD</t>
+          <t>Pintura (interior + exterior)</t>
+        </is>
+      </c>
+      <c r="B14" t="n">
+        <v>968</v>
+      </c>
+      <c r="C14" t="n">
+        <v>726</v>
+      </c>
+      <c r="D14" t="n">
+        <v>-242</v>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>-25%</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Porcelanato premium $32.379/m² → Económico $15.000/m²</t>
-        </is>
-      </c>
-      <c r="B15" t="inlineStr">
-        <is>
-          <t>−54%</t>
-        </is>
-      </c>
-      <c r="C15" t="inlineStr">
-        <is>
-          <t>-1.693 USD</t>
+          <t>Estudio de suelos</t>
+        </is>
+      </c>
+      <c r="B15" t="n">
+        <v>194</v>
+      </c>
+      <c r="C15" t="n">
+        <v>194</v>
+      </c>
+      <c r="D15" t="n">
+        <v>0</v>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>0%</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Puertas interiores $260k → Económicas $95k</t>
-        </is>
-      </c>
-      <c r="B16" t="inlineStr">
-        <is>
-          <t>−63%</t>
-        </is>
-      </c>
-      <c r="C16" t="inlineStr">
-        <is>
-          <t>-495 USD</t>
+          <t>Mesadas</t>
+        </is>
+      </c>
+      <c r="B16" t="n">
+        <v>449</v>
+      </c>
+      <c r="C16" t="n">
+        <v>449</v>
+      </c>
+      <c r="D16" t="n">
+        <v>0</v>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>0%</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Puerta principal $1.900k → Económica $950k</t>
-        </is>
-      </c>
-      <c r="B17" t="inlineStr">
-        <is>
-          <t>−50%</t>
-        </is>
-      </c>
-      <c r="C17" t="inlineStr">
-        <is>
-          <t>-613 USD</t>
+          <t>Mueble cocina (Confort en Aura)</t>
+        </is>
+      </c>
+      <c r="B17" t="n">
+        <v>2452</v>
+      </c>
+      <c r="C17" t="n">
+        <v>0</v>
+      </c>
+      <c r="D17" t="n">
+        <v>-2452</v>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>-100%</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Aberturas $5.000k → Aluminio básico $2.500k</t>
-        </is>
-      </c>
-      <c r="B18" t="inlineStr">
-        <is>
-          <t>−50%</t>
-        </is>
-      </c>
-      <c r="C18" t="inlineStr">
-        <is>
-          <t>-1.613 USD</t>
+          <t>División WPC (duda en Aura)</t>
+        </is>
+      </c>
+      <c r="B18" t="n">
+        <v>340</v>
+      </c>
+      <c r="C18" t="n">
+        <v>0</v>
+      </c>
+      <c r="D18" t="n">
+        <v>-340</v>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>-100%</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Sanitarios $850k+$1.172k → Básicos $1.050k</t>
-        </is>
-      </c>
-      <c r="B19" t="inlineStr">
-        <is>
-          <t>−48%</t>
-        </is>
-      </c>
-      <c r="C19" t="inlineStr">
-        <is>
-          <t>-710 USD</t>
-        </is>
+          <t>Termotanque + cocina + preinst. A/A</t>
+        </is>
+      </c>
+      <c r="B19" t="n">
+        <v>1150</v>
+      </c>
+      <c r="C19" t="n">
+        <v>277</v>
+      </c>
+      <c r="D19" t="n">
+        <v>-873</v>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>-76%</t>
+        </is>
+      </c>
+    </row>
+    <row r="20"/>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>TOTAL MATERIALES</t>
+        </is>
+      </c>
+      <c r="B21" t="n">
+        <v>44135</v>
+      </c>
+      <c r="C21" t="n">
+        <v>33748</v>
+      </c>
+      <c r="D21" t="n">
+        <v>-10387</v>
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="6" t="inlineStr">
-        <is>
-          <t>OBSERVACIONES:</t>
-        </is>
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>Mano de obra (USD 340/m² x 73 m²)</t>
+        </is>
+      </c>
+      <c r="B22" t="n">
+        <v>24820</v>
+      </c>
+      <c r="C22" t="n">
+        <v>24820</v>
+      </c>
+      <c r="D22" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="7" t="inlineStr">
-        <is>
-          <t>• VE es más cara que Aura porque VE incluye finishes completos (terminaciones).</t>
-        </is>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" s="7" t="inlineStr">
-        <is>
-          <t>• Aura Esencial original tiene algunos ítems faltantes/estimados.</t>
-        </is>
-      </c>
-    </row>
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>COSTO DIRECTO</t>
+        </is>
+      </c>
+      <c r="B23" t="n">
+        <v>68955</v>
+      </c>
+      <c r="C23" t="n">
+        <v>58568</v>
+      </c>
+      <c r="D23" t="n">
+        <v>-10387</v>
+      </c>
+    </row>
+    <row r="24"/>
     <row r="25">
-      <c r="A25" s="7" t="inlineStr">
-        <is>
-          <t>• VE tiene especificaciones claras y precios de Mercado Libre (referencias).</t>
-        </is>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" s="7" t="inlineStr">
-        <is>
-          <t>• Ahorro real VE vs Aura está en: siding, techo, pisos, carpinterías.</t>
-        </is>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" s="7" t="inlineStr">
-        <is>
-          <t>• Mano de obra es idéntica (USD 340/m²) en ambos modelos.</t>
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>Nota: precios VE son estimaciones, NO cotizaciones de Mercado Libre; falta validarlos. Aura calculado de Aura_Esencial_Presupuesto_v1.xlsx (incluye ítems Confort y 'duda'; VE los excluye).</t>
         </is>
       </c>
     </row>

</xml_diff>